<commit_message>
Add SOH report for 2026-10-12
</commit_message>
<xml_diff>
--- a/reports/SOH_11_10_2026.xlsx
+++ b/reports/SOH_11_10_2026.xlsx
@@ -7413,7 +7413,7 @@
         </is>
       </c>
       <c r="D253" s="2" t="n">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E253" s="3" t="n">
         <v>8367</v>
@@ -11278,7 +11278,7 @@
         </is>
       </c>
       <c r="D391" s="2" t="n">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="E391" s="3" t="n">
         <v>14934</v>
@@ -13742,7 +13742,7 @@
         </is>
       </c>
       <c r="D479" s="2" t="n">
-        <v>1797</v>
+        <v>1773</v>
       </c>
       <c r="E479" s="3" t="n">
         <v>15262</v>
@@ -13882,7 +13882,7 @@
         </is>
       </c>
       <c r="D484" s="2" t="n">
-        <v>432</v>
+        <v>420</v>
       </c>
       <c r="E484" s="3" t="n">
         <v>5942</v>
@@ -14498,7 +14498,7 @@
         </is>
       </c>
       <c r="D506" s="2" t="n">
-        <v>1245</v>
+        <v>1221</v>
       </c>
       <c r="E506" s="3" t="n">
         <v>8446</v>
@@ -14554,7 +14554,7 @@
         </is>
       </c>
       <c r="D508" s="2" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="E508" s="3" t="n">
         <v>7397</v>
@@ -16458,7 +16458,7 @@
         </is>
       </c>
       <c r="D576" s="2" t="n">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="E576" s="3" t="n">
         <v>16573</v>
@@ -16990,7 +16990,7 @@
         </is>
       </c>
       <c r="D595" s="2" t="n">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="E595" s="3" t="n">
         <v>13111</v>
@@ -17383,7 +17383,7 @@
         </is>
       </c>
       <c r="D609" s="2" t="n">
-        <v>574</v>
+        <v>562</v>
       </c>
       <c r="E609" s="3" t="n">
         <v>8408</v>
@@ -17551,7 +17551,7 @@
         </is>
       </c>
       <c r="D615" s="2" t="n">
-        <v>4063</v>
+        <v>4039</v>
       </c>
       <c r="E615" s="3" t="n">
         <v>10251</v>
@@ -17579,7 +17579,7 @@
         </is>
       </c>
       <c r="D616" s="2" t="n">
-        <v>329</v>
+        <v>305</v>
       </c>
       <c r="E616" s="3" t="n">
         <v>12094</v>
@@ -17719,7 +17719,7 @@
         </is>
       </c>
       <c r="D621" s="2" t="n">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="E621" s="3" t="n">
         <v>8559</v>
@@ -18895,7 +18895,7 @@
         </is>
       </c>
       <c r="D663" s="2" t="n">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="E663" s="3" t="n">
         <v>3987</v>
@@ -19343,7 +19343,7 @@
         </is>
       </c>
       <c r="D679" s="2" t="n">
-        <v>330</v>
+        <v>318</v>
       </c>
       <c r="E679" s="3" t="n">
         <v>2338</v>
@@ -21415,7 +21415,7 @@
         </is>
       </c>
       <c r="D753" s="2" t="n">
-        <v>179</v>
+        <v>155</v>
       </c>
       <c r="E753" s="3" t="n">
         <v>6440</v>
@@ -22115,7 +22115,7 @@
         </is>
       </c>
       <c r="D778" s="2" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E778" s="3" t="n">
         <v>17617</v>
@@ -22815,7 +22815,7 @@
         </is>
       </c>
       <c r="D803" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E803" s="3" t="n">
         <v>11928</v>
@@ -26040,7 +26040,7 @@
         </is>
       </c>
       <c r="D918" s="2" t="n">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="E918" s="3" t="n">
         <v>7700</v>
@@ -28588,7 +28588,7 @@
         </is>
       </c>
       <c r="D1009" s="2" t="n">
-        <v>252</v>
+        <v>246</v>
       </c>
       <c r="E1009" s="3" t="n">
         <v>5243</v>
@@ -29401,7 +29401,7 @@
         </is>
       </c>
       <c r="D1038" s="2" t="n">
-        <v>344</v>
+        <v>340</v>
       </c>
       <c r="E1038" s="3" t="n">
         <v>10480</v>
@@ -29681,7 +29681,7 @@
         </is>
       </c>
       <c r="D1048" s="2" t="n">
-        <v>233</v>
+        <v>221</v>
       </c>
       <c r="E1048" s="3" t="n">
         <v>6142</v>
@@ -30549,7 +30549,7 @@
         </is>
       </c>
       <c r="D1079" s="2" t="n">
-        <v>662</v>
+        <v>656</v>
       </c>
       <c r="E1079" s="3" t="n">
         <v>12935</v>
@@ -30801,7 +30801,7 @@
         </is>
       </c>
       <c r="D1088" s="2" t="n">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="E1088" s="3" t="n">
         <v>15904</v>
@@ -31305,7 +31305,7 @@
         </is>
       </c>
       <c r="D1106" s="2" t="n">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="E1106" s="3" t="n">
         <v>11372</v>
@@ -32733,7 +32733,7 @@
         </is>
       </c>
       <c r="D1157" s="2" t="n">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="E1157" s="3" t="n">
         <v>24480</v>
@@ -32761,7 +32761,7 @@
         </is>
       </c>
       <c r="D1158" s="2" t="n">
-        <v>297</v>
+        <v>249</v>
       </c>
       <c r="E1158" s="3" t="n">
         <v>9174</v>
@@ -33461,7 +33461,7 @@
         </is>
       </c>
       <c r="D1183" s="2" t="n">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E1183" s="3" t="n">
         <v>12865</v>
@@ -33545,7 +33545,7 @@
         </is>
       </c>
       <c r="D1186" s="2" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="E1186" s="3" t="n">
         <v>13709</v>
@@ -34525,7 +34525,7 @@
         </is>
       </c>
       <c r="D1221" s="2" t="n">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="E1221" s="3" t="n">
         <v>15804</v>
@@ -37605,7 +37605,7 @@
         </is>
       </c>
       <c r="D1331" s="2" t="n">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="E1331" s="3" t="n">
         <v>13995</v>
@@ -37717,7 +37717,7 @@
         </is>
       </c>
       <c r="D1335" s="2" t="n">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="E1335" s="3" t="n">
         <v>12005</v>
@@ -38725,7 +38725,7 @@
         </is>
       </c>
       <c r="D1371" s="2" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E1371" s="3" t="n">
         <v>30208</v>
@@ -39481,7 +39481,7 @@
         </is>
       </c>
       <c r="D1398" s="2" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E1398" s="3" t="n">
         <v>5118</v>
@@ -40657,7 +40657,7 @@
         </is>
       </c>
       <c r="D1440" s="2" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E1440" s="3" t="n">
         <v>10733</v>
@@ -41049,7 +41049,7 @@
         </is>
       </c>
       <c r="D1454" s="2" t="n">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="E1454" s="3" t="n">
         <v>12419</v>
@@ -41217,7 +41217,7 @@
         </is>
       </c>
       <c r="D1460" s="2" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E1460" s="3" t="n">
         <v>9428</v>
@@ -41245,7 +41245,7 @@
         </is>
       </c>
       <c r="D1461" s="2" t="n">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="E1461" s="3" t="n">
         <v>11283</v>
@@ -42253,7 +42253,7 @@
         </is>
       </c>
       <c r="D1497" s="2" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="E1497" s="3" t="n">
         <v>37512</v>
@@ -42337,7 +42337,7 @@
         </is>
       </c>
       <c r="D1500" s="2" t="n">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="E1500" s="3" t="n">
         <v>19321</v>
@@ -42379,24 +42379,24 @@
     <row r="1502">
       <c r="A1502" t="inlineStr">
         <is>
-          <t>4894158096239</t>
+          <t>4894158096253</t>
         </is>
       </c>
       <c r="B1502" t="inlineStr">
         <is>
-          <t>PF0648</t>
+          <t>PF0650</t>
         </is>
       </c>
       <c r="C1502" t="inlineStr">
         <is>
-          <t>TRAVEL FEEDER - 300ML</t>
+          <t>TRAVEL FEEDER - 800ML</t>
         </is>
       </c>
       <c r="D1502" s="2" t="n">
-        <v>63</v>
+        <v>28</v>
       </c>
       <c r="E1502" s="3" t="n">
-        <v>9735</v>
+        <v>12491</v>
       </c>
       <c r="F1502" t="inlineStr">
         <is>
@@ -42407,24 +42407,24 @@
     <row r="1503">
       <c r="A1503" t="inlineStr">
         <is>
-          <t>4894158096253</t>
+          <t>9333527593306</t>
         </is>
       </c>
       <c r="B1503" t="inlineStr">
         <is>
-          <t>PF0650</t>
+          <t>AG4194</t>
         </is>
       </c>
       <c r="C1503" t="inlineStr">
         <is>
-          <t>TRAVEL FEEDER - 800ML</t>
+          <t>TRAVEL HANGING TOILETRY BAG</t>
         </is>
       </c>
       <c r="D1503" s="2" t="n">
-        <v>28</v>
+        <v>91</v>
       </c>
       <c r="E1503" s="3" t="n">
-        <v>12491</v>
+        <v>82128</v>
       </c>
       <c r="F1503" t="inlineStr">
         <is>
@@ -42435,24 +42435,24 @@
     <row r="1504">
       <c r="A1504" t="inlineStr">
         <is>
-          <t>9333527593306</t>
+          <t>9333527811240</t>
         </is>
       </c>
       <c r="B1504" t="inlineStr">
         <is>
-          <t>AG4194</t>
+          <t>RM0000011</t>
         </is>
       </c>
       <c r="C1504" t="inlineStr">
         <is>
-          <t>TRAVEL HANGING TOILETRY BAG</t>
+          <t>TRAVEL LOTION &amp; SPRAY 3 BOTTLE SET 50ML 50ML 100ML</t>
         </is>
       </c>
       <c r="D1504" s="2" t="n">
-        <v>91</v>
+        <v>17</v>
       </c>
       <c r="E1504" s="3" t="n">
-        <v>82128</v>
+        <v>28056</v>
       </c>
       <c r="F1504" t="inlineStr">
         <is>
@@ -42463,24 +42463,24 @@
     <row r="1505">
       <c r="A1505" t="inlineStr">
         <is>
-          <t>9333527811240</t>
+          <t>9333527176394</t>
         </is>
       </c>
       <c r="B1505" t="inlineStr">
         <is>
-          <t>RM0000011</t>
+          <t>OB0083</t>
         </is>
       </c>
       <c r="C1505" t="inlineStr">
         <is>
-          <t>TRAVEL LOTION &amp; SPRAY 3 BOTTLE SET 50ML 50ML 100ML</t>
+          <t>TRAVEL MUG CER. W/SILICON GRIP</t>
         </is>
       </c>
       <c r="D1505" s="2" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="E1505" s="3" t="n">
-        <v>28056</v>
+        <v>19001</v>
       </c>
       <c r="F1505" t="inlineStr">
         <is>
@@ -42491,24 +42491,24 @@
     <row r="1506">
       <c r="A1506" t="inlineStr">
         <is>
-          <t>9333527176394</t>
+          <t>9333527610607</t>
         </is>
       </c>
       <c r="B1506" t="inlineStr">
         <is>
-          <t>OB0083</t>
+          <t>RG0292</t>
         </is>
       </c>
       <c r="C1506" t="inlineStr">
         <is>
-          <t>TRAVEL MUG CER. W/SILICON GRIP</t>
+          <t>TRAVEL MUG DOUBLE WALLED 473ML</t>
         </is>
       </c>
       <c r="D1506" s="2" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E1506" s="3" t="n">
-        <v>19001</v>
+        <v>27542</v>
       </c>
       <c r="F1506" t="inlineStr">
         <is>
@@ -42519,24 +42519,24 @@
     <row r="1507">
       <c r="A1507" t="inlineStr">
         <is>
-          <t>9333527610607</t>
+          <t>4894158096239</t>
         </is>
       </c>
       <c r="B1507" t="inlineStr">
         <is>
-          <t>RG0292</t>
+          <t>PF0648</t>
         </is>
       </c>
       <c r="C1507" t="inlineStr">
         <is>
-          <t>TRAVEL MUG DOUBLE WALLED 473ML</t>
+          <t>TRAVEL FEEDER - 300ML</t>
         </is>
       </c>
       <c r="D1507" s="2" t="n">
-        <v>30</v>
+        <v>63</v>
       </c>
       <c r="E1507" s="3" t="n">
-        <v>27542</v>
+        <v>9735</v>
       </c>
       <c r="F1507" t="inlineStr">
         <is>
@@ -42842,7 +42842,7 @@
         </is>
       </c>
       <c r="D1518" s="2" t="n">
-        <v>332</v>
+        <v>322</v>
       </c>
       <c r="E1518" s="3" t="n">
         <v>6000</v>
@@ -43710,7 +43710,7 @@
         </is>
       </c>
       <c r="D1549" s="2" t="n">
-        <v>269</v>
+        <v>263</v>
       </c>
       <c r="E1549" s="3" t="n">
         <v>11129</v>
@@ -44383,7 +44383,7 @@
         </is>
       </c>
       <c r="D1573" s="2" t="n">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="E1573" s="3" t="n">
         <v>15682</v>

</xml_diff>